<commit_message>
temp - creating better manifest for testing and template
</commit_message>
<xml_diff>
--- a/EVE_WORK/tests_monitoring/1_test_data_ST22_dummy.xlsx
+++ b/EVE_WORK/tests_monitoring/1_test_data_ST22_dummy.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t xml:space="preserve">data_schema_id (raw data)</t>
   </si>
@@ -35,6 +35,33 @@
     <t xml:space="preserve">origin (raw data)</t>
   </si>
   <si>
+    <t xml:space="preserve">comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input_fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input_fields Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wrangling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wrangling status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">output_fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">output_fields status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comments</t>
+  </si>
+  <si>
     <t xml:space="preserve">Summary</t>
   </si>
   <si>
@@ -42,6 +69,30 @@
   </si>
   <si>
     <t xml:space="preserve">default Abromics pipeline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mirrored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary_input_fields.yaml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summary_quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no need</t>
+  </si>
+  <si>
+    <t xml:space="preserve">summary_quality_output_fields.yaml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selection columns via output fields</t>
   </si>
   <si>
     <t xml:space="preserve">Quality_metrics</t>
@@ -126,20 +177,51 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFD7"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FF969696"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEDCE6"/>
+        <bgColor rgb="FFDDE8CB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE8CB"/>
+        <bgColor rgb="FFDEDCE6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -168,12 +250,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -186,6 +288,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFD7"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFDEDCE6"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFDDE8CB"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF81D41A"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -300,144 +462,230 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="29.35"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="3" width="16.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="4" width="17.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="4" width="20.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="5" width="24.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="5" width="22.4"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="12" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>5</v>
+      <c r="A2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>5</v>
+      <c r="A3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>5</v>
+      <c r="A4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>5</v>
+      <c r="A5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>5</v>
+      <c r="A6" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>5</v>
+      <c r="A7" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>5</v>
+      <c r="A8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
+      <c r="A9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>29</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>20</v>
+      <c r="A11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -461,7 +709,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement persona-based UI reactivity tests and consolidate architectural documentation and tasks
</commit_message>
<xml_diff>
--- a/EVE_WORK/tests_monitoring/1_test_data_ST22_dummy.xlsx
+++ b/EVE_WORK/tests_monitoring/1_test_data_ST22_dummy.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
   <si>
     <t xml:space="preserve">data_schema_id (raw data)</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t xml:space="preserve">Quality_metrics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEACTIVATED</t>
   </si>
   <si>
     <t xml:space="preserve">Detailed_summary</t>
@@ -588,43 +591,55 @@
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>13</v>
@@ -635,7 +650,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>13</v>
@@ -646,7 +661,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>13</v>
@@ -657,35 +672,35 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -709,7 +724,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>